<commit_message>
Add messaging functionality with Twilio and Telegram integration; update UI and requirements
</commit_message>
<xml_diff>
--- a/weighment_data.xlsx
+++ b/weighment_data.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G2"/>
+  <dimension ref="A1:R8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -439,15 +439,70 @@
       </c>
       <c r="E1" t="inlineStr">
         <is>
+          <t>Challan</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Customer Code</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Customer Name</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Product Code</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>Product Name</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>Source Code</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>Source Name</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>Destination Code</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>Destination Name</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>Transporter Code</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>Transporter Name</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
           <t>Gross Weight</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>Tare Weight</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>Net Weight</t>
         </is>
@@ -480,6 +535,510 @@
       </c>
       <c r="G2" t="n">
         <v>-9189</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>dkhcbdvcfkh</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>15-04-2026</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>19:35:42</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>cdcd</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>kjdhchd</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>jhhdfjhdsg</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>hjgdfdfhd</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>jhgdjhdsg</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>jhdfjhdjhd</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>kjscbkb</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>s</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>kjhs</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>s</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>s</t>
+        </is>
+      </c>
+      <c r="P3" t="n">
+        <v>21835</v>
+      </c>
+      <c r="Q3" t="n">
+        <v>32460</v>
+      </c>
+      <c r="R3" t="n">
+        <v>-10625</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>dwjhd</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>15-04-2026</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>19:42:20</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>jsdd</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>sjvh</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>s</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>kjs</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>ss</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>ss</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>s</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>ss</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>ss</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>ss</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>ss</t>
+        </is>
+      </c>
+      <c r="P4" t="n">
+        <v>3886</v>
+      </c>
+      <c r="Q4" t="n">
+        <v>6415</v>
+      </c>
+      <c r="R4" t="n">
+        <v>-2529</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>hgfhgf</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>15-04-2026</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>19:53:31</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>jg</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>kgh</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>khg</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>hjg</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>jhg</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>jh</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>jhg</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>jhg</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>hf</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>ghf</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>jh</t>
+        </is>
+      </c>
+      <c r="P5" t="n">
+        <v>8149</v>
+      </c>
+      <c r="Q5" t="n">
+        <v>15144</v>
+      </c>
+      <c r="R5" t="n">
+        <v>-6995</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>hj</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>15-04-2026</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>19:54:01</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>jhg</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>jgjh</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>dd</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>dd</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>ff</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>ff</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>ff</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>ff</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>ff</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>ff</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>ff</t>
+        </is>
+      </c>
+      <c r="P6" t="n">
+        <v>3916</v>
+      </c>
+      <c r="Q6" t="n">
+        <v>42022</v>
+      </c>
+      <c r="R6" t="n">
+        <v>-38106</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>hj</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>15-04-2026</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>20:00:45</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>jhjh</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>jhg</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>kj</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>hj</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>jhg</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>gf</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>jhf</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>ngf</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>hjf</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>ghf</t>
+        </is>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>hdf</t>
+        </is>
+      </c>
+      <c r="P7" t="n">
+        <v>47243</v>
+      </c>
+      <c r="Q7" t="n">
+        <v>49539</v>
+      </c>
+      <c r="R7" t="n">
+        <v>-2296</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>jfdhd</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>15-04-2026</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>20:22:53</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>ss</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>ssss</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>hddhd</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>sss</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>ddddd</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>hhs</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>ddd</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>dd</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>dd</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>dd</t>
+        </is>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>dd</t>
+        </is>
+      </c>
+      <c r="P8" t="n">
+        <v>27091</v>
+      </c>
+      <c r="Q8" t="n">
+        <v>19829</v>
+      </c>
+      <c r="R8" t="n">
+        <v>7262</v>
       </c>
     </row>
   </sheetData>

</xml_diff>